<commit_message>
added email jenkins settings
</commit_message>
<xml_diff>
--- a/testsheets/TestSuite.xlsx
+++ b/testsheets/TestSuite.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\keyword_excel_framework\testsheets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8B93DE9-5FB2-4227-B03C-BD7B94BDD3C6}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AE1A297-0171-4DB0-9927-1587DBE4D7F7}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7425" tabRatio="811" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7425" tabRatio="811" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TestSteps" sheetId="1" r:id="rId1"/>
@@ -1210,7 +1210,7 @@
         <v>20</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>22</v>

</xml_diff>